<commit_message>
fix: F&B 500 (esquema columnas) + pre-filtro conservador
1. F&B ERROR 500 RESUELTO:
   Causa raíz: los datos demo F&B usaban nombres de columna distintos
   a los que tab_fb_dashboard.py espera. El groupby(['id_receta',
   'nombre_plato']) crasheaba porque la columna se llamaba 'plato'.
   FIX: regenerados recetas/inventario/ventas/mermas con el esquema
   EXACTO: ingredientes_json, nombre_plato, coste_merma, etc.
   Verificado: total €61,773, 8 recetas, FC% 13.5%, groupby OK.

2. PRE-FILTRO MÁS CONSERVADOR:
   GRUPA EVENT (depósito) y 2521-5 se rechazaban antes de llegar
   a Claude. El filtro de contenido era muy agresivo.
   FIX: solo bloquea con señales MUY claras de no-factura.
   Añadidas señales de factura: deposit, depósito, anticipo,
   proforma, iban, subtotal, importe, amount, €, eur, fee.
   En duda → deja pasar a Claude (mejor juez).
</commit_message>
<xml_diff>
--- a/datos-referencia/inventario.xlsx
+++ b/datos-referencia/inventario.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Inventario" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -413,43 +413,43 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G6"/>
+  <dimension ref="A1:G20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>producto</t>
+          <t>ingrediente</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>categoria</t>
+          <t>coste_unitario</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>cantidad</t>
+          <t>stock_actual_kg_l</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
+          <t>stock_inicial_kg_l</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
           <t>unidad</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>precio_unitario</t>
-        </is>
-      </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>valor_total</t>
+          <t>proveedor</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
         <is>
-          <t>minimo</t>
+          <t>critico</t>
         </is>
       </c>
     </row>
@@ -459,143 +459,549 @@
           <t>Lubina fresca</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Pescados</t>
-        </is>
+      <c r="B2" t="n">
+        <v>18</v>
       </c>
       <c r="C2" t="n">
-        <v>45</v>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>kg</t>
-        </is>
-      </c>
-      <c r="E2" t="n">
-        <v>18</v>
-      </c>
-      <c r="F2" t="n">
-        <v>810</v>
-      </c>
-      <c r="G2" t="n">
-        <v>20</v>
+        <v>24.8</v>
+      </c>
+      <c r="D2" t="n">
+        <v>47.5</v>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Proveedor Lubina f</t>
+        </is>
+      </c>
+      <c r="G2" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Entrecot</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Carnes</t>
-        </is>
+          <t>Sal marina</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>1.2</v>
       </c>
       <c r="C3" t="n">
-        <v>30</v>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>kg</t>
-        </is>
-      </c>
-      <c r="E3" t="n">
-        <v>22</v>
-      </c>
-      <c r="F3" t="n">
-        <v>660</v>
-      </c>
-      <c r="G3" t="n">
-        <v>15</v>
+        <v>10.6</v>
+      </c>
+      <c r="D3" t="n">
+        <v>22.9</v>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Proveedor Sal mari</t>
+        </is>
+      </c>
+      <c r="G3" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Arroz bomba</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Arroces</t>
-        </is>
+          <t>Aceite oliva</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>8</v>
       </c>
       <c r="C4" t="n">
-        <v>50</v>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>kg</t>
-        </is>
-      </c>
-      <c r="E4" t="n">
-        <v>3.2</v>
-      </c>
-      <c r="F4" t="n">
-        <v>160</v>
-      </c>
-      <c r="G4" t="n">
-        <v>20</v>
+        <v>22</v>
+      </c>
+      <c r="D4" t="n">
+        <v>48.9</v>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Proveedor Aceite o</t>
+        </is>
+      </c>
+      <c r="G4" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Trufa negra</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Especias</t>
-        </is>
+          <t>Entrecot</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>22</v>
       </c>
       <c r="C5" t="n">
-        <v>2</v>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>kg</t>
-        </is>
-      </c>
-      <c r="E5" t="n">
-        <v>180</v>
-      </c>
-      <c r="F5" t="n">
-        <v>360</v>
-      </c>
-      <c r="G5" t="n">
-        <v>1</v>
+        <v>35.3</v>
+      </c>
+      <c r="D5" t="n">
+        <v>58.3</v>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Proveedor Entrecot</t>
+        </is>
+      </c>
+      <c r="G5" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
+          <t>Patata</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="C6" t="n">
+        <v>14.2</v>
+      </c>
+      <c r="D6" t="n">
+        <v>24.3</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Proveedor Patata</t>
+        </is>
+      </c>
+      <c r="G6" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Mantequilla</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>9</v>
+      </c>
+      <c r="C7" t="n">
+        <v>31.3</v>
+      </c>
+      <c r="D7" t="n">
+        <v>55.9</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Proveedor Mantequi</t>
+        </is>
+      </c>
+      <c r="G7" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Arroz bomba</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="C8" t="n">
+        <v>26</v>
+      </c>
+      <c r="D8" t="n">
+        <v>44.5</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Proveedor Arroz bo</t>
+        </is>
+      </c>
+      <c r="G8" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Trufa negra</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>180</v>
+      </c>
+      <c r="C9" t="n">
+        <v>15.5</v>
+      </c>
+      <c r="D9" t="n">
+        <v>34.8</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Proveedor Trufa ne</t>
+        </is>
+      </c>
+      <c r="G9" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Parmesano</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>15</v>
+      </c>
+      <c r="C10" t="n">
+        <v>11.9</v>
+      </c>
+      <c r="D10" t="n">
+        <v>31.6</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Proveedor Parmesan</t>
+        </is>
+      </c>
+      <c r="G10" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Lechuga</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>2</v>
+      </c>
+      <c r="C11" t="n">
+        <v>35</v>
+      </c>
+      <c r="D11" t="n">
+        <v>51.3</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Proveedor Lechuga</t>
+        </is>
+      </c>
+      <c r="G11" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Pollo</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>6.5</v>
+      </c>
+      <c r="C12" t="n">
+        <v>12.5</v>
+      </c>
+      <c r="D12" t="n">
+        <v>36</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Proveedor Pollo</t>
+        </is>
+      </c>
+      <c r="G12" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
           <t>Chocolate 70%</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Postres</t>
-        </is>
-      </c>
-      <c r="C6" t="n">
-        <v>15</v>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>kg</t>
-        </is>
-      </c>
-      <c r="E6" t="n">
+      <c r="B13" t="n">
         <v>12</v>
       </c>
-      <c r="F6" t="n">
-        <v>180</v>
-      </c>
-      <c r="G6" t="n">
-        <v>5</v>
+      <c r="C13" t="n">
+        <v>42.2</v>
+      </c>
+      <c r="D13" t="n">
+        <v>59.5</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Proveedor Chocolat</t>
+        </is>
+      </c>
+      <c r="G13" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Harina</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>1</v>
+      </c>
+      <c r="C14" t="n">
+        <v>19.5</v>
+      </c>
+      <c r="D14" t="n">
+        <v>35.8</v>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Proveedor Harina</t>
+        </is>
+      </c>
+      <c r="G14" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Huevo</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>3</v>
+      </c>
+      <c r="C15" t="n">
+        <v>18.6</v>
+      </c>
+      <c r="D15" t="n">
+        <v>31.7</v>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Proveedor Huevo</t>
+        </is>
+      </c>
+      <c r="G15" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Marisco</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>14</v>
+      </c>
+      <c r="C16" t="n">
+        <v>9.5</v>
+      </c>
+      <c r="D16" t="n">
+        <v>23.4</v>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Proveedor Marisco</t>
+        </is>
+      </c>
+      <c r="G16" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Tomate</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="C17" t="n">
+        <v>9.800000000000001</v>
+      </c>
+      <c r="D17" t="n">
+        <v>25.9</v>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Proveedor Tomate</t>
+        </is>
+      </c>
+      <c r="G17" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Carne picada</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>9.5</v>
+      </c>
+      <c r="C18" t="n">
+        <v>17.6</v>
+      </c>
+      <c r="D18" t="n">
+        <v>22.9</v>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>Proveedor Carne pi</t>
+        </is>
+      </c>
+      <c r="G18" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Pan brioche</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>3</v>
+      </c>
+      <c r="C19" t="n">
+        <v>25.7</v>
+      </c>
+      <c r="D19" t="n">
+        <v>41.1</v>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>Proveedor Pan brio</t>
+        </is>
+      </c>
+      <c r="G19" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Queso</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>12</v>
+      </c>
+      <c r="C20" t="n">
+        <v>29</v>
+      </c>
+      <c r="D20" t="n">
+        <v>39.8</v>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Proveedor Queso</t>
+        </is>
+      </c>
+      <c r="G20" t="b">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix: inventario y mermas F&B — añadir columna 'categoria' y 'unidad'
Las subpestañas Inventario y Mermas daban 'Error inventario' (500)
porque los datos demo no tenían la columna 'categoria' que el código
espera (api_inventario y api_mermas la usan).

Regenerados con TODAS las columnas:
- inventario: ingrediente, categoria, coste_unitario, stock_actual_kg_l,
  stock_inicial_kg_l, unidad, proveedor, critico (19 items)
- mermas: fecha, ingrediente, categoria, cantidad_merma, unidad, causa,
  coste_unitario, coste_merma (10 registros, 4 categorías)

Verificado localmente: ambos endpoints procesan sin error.
Resumen F&B ya funcionaba (€61.773, FC% 14.49%).
</commit_message>
<xml_diff>
--- a/datos-referencia/inventario.xlsx
+++ b/datos-referencia/inventario.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G20"/>
+  <dimension ref="A1:H20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -424,30 +424,35 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
+          <t>categoria</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
           <t>coste_unitario</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>stock_actual_kg_l</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>stock_inicial_kg_l</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>unidad</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>proveedor</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>critico</t>
         </is>
@@ -459,26 +464,31 @@
           <t>Lubina fresca</t>
         </is>
       </c>
-      <c r="B2" t="n">
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Pescados</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
         <v>18</v>
       </c>
-      <c r="C2" t="n">
-        <v>24.8</v>
-      </c>
       <c r="D2" t="n">
-        <v>47.5</v>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>kg</t>
-        </is>
+        <v>10.8</v>
+      </c>
+      <c r="E2" t="n">
+        <v>33.5</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Proveedor Lubina f</t>
-        </is>
-      </c>
-      <c r="G2" t="b">
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Distribuciones Pescados</t>
+        </is>
+      </c>
+      <c r="H2" t="b">
         <v>0</v>
       </c>
     </row>
@@ -488,26 +498,31 @@
           <t>Sal marina</t>
         </is>
       </c>
-      <c r="B3" t="n">
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Condimentos</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
         <v>1.2</v>
       </c>
-      <c r="C3" t="n">
-        <v>10.6</v>
-      </c>
       <c r="D3" t="n">
-        <v>22.9</v>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>kg</t>
-        </is>
+        <v>15</v>
+      </c>
+      <c r="E3" t="n">
+        <v>27.7</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Proveedor Sal mari</t>
-        </is>
-      </c>
-      <c r="G3" t="b">
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Distribuciones Condimentos</t>
+        </is>
+      </c>
+      <c r="H3" t="b">
         <v>0</v>
       </c>
     </row>
@@ -517,26 +532,31 @@
           <t>Aceite oliva</t>
         </is>
       </c>
-      <c r="B4" t="n">
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Aceites</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
         <v>8</v>
       </c>
-      <c r="C4" t="n">
-        <v>22</v>
-      </c>
       <c r="D4" t="n">
+        <v>16.2</v>
+      </c>
+      <c r="E4" t="n">
         <v>48.9</v>
       </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>kg</t>
-        </is>
-      </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Proveedor Aceite o</t>
-        </is>
-      </c>
-      <c r="G4" t="b">
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Distribuciones Aceites</t>
+        </is>
+      </c>
+      <c r="H4" t="b">
         <v>0</v>
       </c>
     </row>
@@ -546,26 +566,31 @@
           <t>Entrecot</t>
         </is>
       </c>
-      <c r="B5" t="n">
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Carnes</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
         <v>22</v>
       </c>
-      <c r="C5" t="n">
-        <v>35.3</v>
-      </c>
       <c r="D5" t="n">
-        <v>58.3</v>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>kg</t>
-        </is>
+        <v>16.6</v>
+      </c>
+      <c r="E5" t="n">
+        <v>56.6</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Proveedor Entrecot</t>
-        </is>
-      </c>
-      <c r="G5" t="b">
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Distribuciones Carnes</t>
+        </is>
+      </c>
+      <c r="H5" t="b">
         <v>0</v>
       </c>
     </row>
@@ -575,26 +600,31 @@
           <t>Patata</t>
         </is>
       </c>
-      <c r="B6" t="n">
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Verduras</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
         <v>1.5</v>
       </c>
-      <c r="C6" t="n">
-        <v>14.2</v>
-      </c>
       <c r="D6" t="n">
-        <v>24.3</v>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>kg</t>
-        </is>
+        <v>12.6</v>
+      </c>
+      <c r="E6" t="n">
+        <v>55.4</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Proveedor Patata</t>
-        </is>
-      </c>
-      <c r="G6" t="b">
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Distribuciones Verduras</t>
+        </is>
+      </c>
+      <c r="H6" t="b">
         <v>0</v>
       </c>
     </row>
@@ -604,26 +634,31 @@
           <t>Mantequilla</t>
         </is>
       </c>
-      <c r="B7" t="n">
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Lácteos</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
         <v>9</v>
       </c>
-      <c r="C7" t="n">
-        <v>31.3</v>
-      </c>
       <c r="D7" t="n">
-        <v>55.9</v>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>kg</t>
-        </is>
+        <v>16.5</v>
+      </c>
+      <c r="E7" t="n">
+        <v>37.3</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Proveedor Mantequi</t>
-        </is>
-      </c>
-      <c r="G7" t="b">
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Distribuciones Lácteos</t>
+        </is>
+      </c>
+      <c r="H7" t="b">
         <v>0</v>
       </c>
     </row>
@@ -633,26 +668,31 @@
           <t>Arroz bomba</t>
         </is>
       </c>
-      <c r="B8" t="n">
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Cereales</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
         <v>3.2</v>
       </c>
-      <c r="C8" t="n">
-        <v>26</v>
-      </c>
       <c r="D8" t="n">
-        <v>44.5</v>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>kg</t>
-        </is>
+        <v>18.2</v>
+      </c>
+      <c r="E8" t="n">
+        <v>51.3</v>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Proveedor Arroz bo</t>
-        </is>
-      </c>
-      <c r="G8" t="b">
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Distribuciones Cereales</t>
+        </is>
+      </c>
+      <c r="H8" t="b">
         <v>0</v>
       </c>
     </row>
@@ -662,26 +702,31 @@
           <t>Trufa negra</t>
         </is>
       </c>
-      <c r="B9" t="n">
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Especias</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
         <v>180</v>
       </c>
-      <c r="C9" t="n">
-        <v>15.5</v>
-      </c>
       <c r="D9" t="n">
-        <v>34.8</v>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>kg</t>
-        </is>
+        <v>19.8</v>
+      </c>
+      <c r="E9" t="n">
+        <v>23.9</v>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Proveedor Trufa ne</t>
-        </is>
-      </c>
-      <c r="G9" t="b">
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Distribuciones Especias</t>
+        </is>
+      </c>
+      <c r="H9" t="b">
         <v>0</v>
       </c>
     </row>
@@ -691,27 +736,32 @@
           <t>Parmesano</t>
         </is>
       </c>
-      <c r="B10" t="n">
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Lácteos</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
         <v>15</v>
       </c>
-      <c r="C10" t="n">
-        <v>11.9</v>
-      </c>
       <c r="D10" t="n">
-        <v>31.6</v>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>kg</t>
-        </is>
+        <v>33.2</v>
+      </c>
+      <c r="E10" t="n">
+        <v>47.8</v>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Proveedor Parmesan</t>
-        </is>
-      </c>
-      <c r="G10" t="b">
-        <v>1</v>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Distribuciones Lácteos</t>
+        </is>
+      </c>
+      <c r="H10" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="11">
@@ -720,26 +770,31 @@
           <t>Lechuga</t>
         </is>
       </c>
-      <c r="B11" t="n">
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Verduras</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
         <v>2</v>
       </c>
-      <c r="C11" t="n">
-        <v>35</v>
-      </c>
       <c r="D11" t="n">
-        <v>51.3</v>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>kg</t>
-        </is>
+        <v>6.7</v>
+      </c>
+      <c r="E11" t="n">
+        <v>24.9</v>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Proveedor Lechuga</t>
-        </is>
-      </c>
-      <c r="G11" t="b">
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>Distribuciones Verduras</t>
+        </is>
+      </c>
+      <c r="H11" t="b">
         <v>0</v>
       </c>
     </row>
@@ -749,27 +804,32 @@
           <t>Pollo</t>
         </is>
       </c>
-      <c r="B12" t="n">
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Carnes</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
         <v>6.5</v>
       </c>
-      <c r="C12" t="n">
-        <v>12.5</v>
-      </c>
       <c r="D12" t="n">
-        <v>36</v>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>kg</t>
-        </is>
+        <v>22.6</v>
+      </c>
+      <c r="E12" t="n">
+        <v>43.4</v>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Proveedor Pollo</t>
-        </is>
-      </c>
-      <c r="G12" t="b">
-        <v>1</v>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>Distribuciones Carnes</t>
+        </is>
+      </c>
+      <c r="H12" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="13">
@@ -778,26 +838,31 @@
           <t>Chocolate 70%</t>
         </is>
       </c>
-      <c r="B13" t="n">
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Reposteria</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
         <v>12</v>
       </c>
-      <c r="C13" t="n">
-        <v>42.2</v>
-      </c>
       <c r="D13" t="n">
-        <v>59.5</v>
-      </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>kg</t>
-        </is>
+        <v>9.5</v>
+      </c>
+      <c r="E13" t="n">
+        <v>24.9</v>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Proveedor Chocolat</t>
-        </is>
-      </c>
-      <c r="G13" t="b">
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>Distribuciones Reposteria</t>
+        </is>
+      </c>
+      <c r="H13" t="b">
         <v>0</v>
       </c>
     </row>
@@ -807,26 +872,31 @@
           <t>Harina</t>
         </is>
       </c>
-      <c r="B14" t="n">
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Cereales</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
         <v>1</v>
       </c>
-      <c r="C14" t="n">
-        <v>19.5</v>
-      </c>
       <c r="D14" t="n">
-        <v>35.8</v>
-      </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>kg</t>
-        </is>
+        <v>29</v>
+      </c>
+      <c r="E14" t="n">
+        <v>36</v>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Proveedor Harina</t>
-        </is>
-      </c>
-      <c r="G14" t="b">
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>Distribuciones Cereales</t>
+        </is>
+      </c>
+      <c r="H14" t="b">
         <v>0</v>
       </c>
     </row>
@@ -836,26 +906,31 @@
           <t>Huevo</t>
         </is>
       </c>
-      <c r="B15" t="n">
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Lácteos</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
         <v>3</v>
       </c>
-      <c r="C15" t="n">
-        <v>18.6</v>
-      </c>
       <c r="D15" t="n">
-        <v>31.7</v>
-      </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>kg</t>
-        </is>
+        <v>33.6</v>
+      </c>
+      <c r="E15" t="n">
+        <v>50.4</v>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Proveedor Huevo</t>
-        </is>
-      </c>
-      <c r="G15" t="b">
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>Distribuciones Lácteos</t>
+        </is>
+      </c>
+      <c r="H15" t="b">
         <v>0</v>
       </c>
     </row>
@@ -865,26 +940,31 @@
           <t>Marisco</t>
         </is>
       </c>
-      <c r="B16" t="n">
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Pescados</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
         <v>14</v>
       </c>
-      <c r="C16" t="n">
-        <v>9.5</v>
-      </c>
       <c r="D16" t="n">
-        <v>23.4</v>
-      </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>kg</t>
-        </is>
+        <v>11.2</v>
+      </c>
+      <c r="E16" t="n">
+        <v>26.4</v>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Proveedor Marisco</t>
-        </is>
-      </c>
-      <c r="G16" t="b">
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>Distribuciones Pescados</t>
+        </is>
+      </c>
+      <c r="H16" t="b">
         <v>0</v>
       </c>
     </row>
@@ -894,27 +974,32 @@
           <t>Tomate</t>
         </is>
       </c>
-      <c r="B17" t="n">
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Verduras</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
         <v>2.5</v>
       </c>
-      <c r="C17" t="n">
-        <v>9.800000000000001</v>
-      </c>
       <c r="D17" t="n">
-        <v>25.9</v>
-      </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>kg</t>
-        </is>
+        <v>21.5</v>
+      </c>
+      <c r="E17" t="n">
+        <v>43.2</v>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Proveedor Tomate</t>
-        </is>
-      </c>
-      <c r="G17" t="b">
-        <v>1</v>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>Distribuciones Verduras</t>
+        </is>
+      </c>
+      <c r="H17" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="18">
@@ -923,26 +1008,31 @@
           <t>Carne picada</t>
         </is>
       </c>
-      <c r="B18" t="n">
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Carnes</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
         <v>9.5</v>
       </c>
-      <c r="C18" t="n">
-        <v>17.6</v>
-      </c>
       <c r="D18" t="n">
-        <v>22.9</v>
-      </c>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>kg</t>
-        </is>
+        <v>27.2</v>
+      </c>
+      <c r="E18" t="n">
+        <v>49</v>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Proveedor Carne pi</t>
-        </is>
-      </c>
-      <c r="G18" t="b">
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>Distribuciones Carnes</t>
+        </is>
+      </c>
+      <c r="H18" t="b">
         <v>0</v>
       </c>
     </row>
@@ -952,26 +1042,31 @@
           <t>Pan brioche</t>
         </is>
       </c>
-      <c r="B19" t="n">
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Panaderia</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
         <v>3</v>
       </c>
-      <c r="C19" t="n">
-        <v>25.7</v>
-      </c>
       <c r="D19" t="n">
-        <v>41.1</v>
-      </c>
-      <c r="E19" t="inlineStr">
-        <is>
-          <t>kg</t>
-        </is>
+        <v>18.2</v>
+      </c>
+      <c r="E19" t="n">
+        <v>34</v>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Proveedor Pan brio</t>
-        </is>
-      </c>
-      <c r="G19" t="b">
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>Distribuciones Panaderia</t>
+        </is>
+      </c>
+      <c r="H19" t="b">
         <v>0</v>
       </c>
     </row>
@@ -981,26 +1076,31 @@
           <t>Queso</t>
         </is>
       </c>
-      <c r="B20" t="n">
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Lácteos</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
         <v>12</v>
       </c>
-      <c r="C20" t="n">
-        <v>29</v>
-      </c>
       <c r="D20" t="n">
-        <v>39.8</v>
-      </c>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t>kg</t>
-        </is>
+        <v>5.6</v>
+      </c>
+      <c r="E20" t="n">
+        <v>22</v>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Proveedor Queso</t>
-        </is>
-      </c>
-      <c r="G20" t="b">
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>Distribuciones Lácteos</t>
+        </is>
+      </c>
+      <c r="H20" t="b">
         <v>0</v>
       </c>
     </row>

</xml_diff>